<commit_message>
Add Physics data and earnings footnote to salary page
Workbook gains a Physics tab (96 universities), reflected in the
regenerated charts. The shareable page adds a footnote explaining that
earnings are median IRS-reported incomes for 2017-18 and 2018-19
graduates. Remove the static PNG.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/NYT_EE.xlsx
+++ b/Data/NYT_EE.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bobbass\GitHubLocal\NYT-Engineering-Salaries\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EC82407-6797-4DE7-A845-8631D975FA66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B010C64-FF7F-4BC8-A6D4-7BAC16CE7F79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="800" windowWidth="38620" windowHeight="21100" activeTab="3" xr2:uid="{E272B9CE-C2EB-4DBE-9828-72CD11372EDF}"/>
+    <workbookView xWindow="-38510" yWindow="800" windowWidth="38620" windowHeight="21100" activeTab="4" xr2:uid="{E272B9CE-C2EB-4DBE-9828-72CD11372EDF}"/>
   </bookViews>
   <sheets>
     <sheet name="Electrical Engineering" sheetId="1" r:id="rId1"/>
     <sheet name="Mechancial Engineering" sheetId="2" r:id="rId2"/>
     <sheet name="Civil Engineering" sheetId="3" r:id="rId3"/>
     <sheet name="Computer Science" sheetId="4" r:id="rId4"/>
+    <sheet name="Physics" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1080" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1178" uniqueCount="504">
   <si>
     <t>UNIVERSITY</t>
   </si>
@@ -1485,6 +1486,75 @@
   </si>
   <si>
     <t>Fayetteville State University</t>
+  </si>
+  <si>
+    <t>College of the Holy Cross</t>
+  </si>
+  <si>
+    <t>Le Moyne College</t>
+  </si>
+  <si>
+    <t>Shippensburg University of Pennsylvania</t>
+  </si>
+  <si>
+    <t>Southern Arkansas University Main Campus</t>
+  </si>
+  <si>
+    <t>West Virginia Wesleyan College</t>
+  </si>
+  <si>
+    <t>University of Wisconsin-Eau Claire</t>
+  </si>
+  <si>
+    <t>Stockton University</t>
+  </si>
+  <si>
+    <t>Bethel University (Minnesota)</t>
+  </si>
+  <si>
+    <t>University of Wisconsin-River Falls</t>
+  </si>
+  <si>
+    <t>University of Wisconsin-La Crosse</t>
+  </si>
+  <si>
+    <t>SUNY Oneonta</t>
+  </si>
+  <si>
+    <t>Salisbury University</t>
+  </si>
+  <si>
+    <t>Seton Hall University</t>
+  </si>
+  <si>
+    <t>SUNY College at Geneseo</t>
+  </si>
+  <si>
+    <t>University of Oregon</t>
+  </si>
+  <si>
+    <t>Kutztown University of Pennsylvania</t>
+  </si>
+  <si>
+    <t>Gustavus Adolphus College</t>
+  </si>
+  <si>
+    <t>University of Northern Colorado</t>
+  </si>
+  <si>
+    <t>St. John's University (New York)</t>
+  </si>
+  <si>
+    <t>Siena College</t>
+  </si>
+  <si>
+    <t>Indiana University of Pennsylvania-Main Campus</t>
+  </si>
+  <si>
+    <t>Morehead State University</t>
+  </si>
+  <si>
+    <t>Coe College</t>
   </si>
 </sst>
 </file>
@@ -10509,4 +10579,790 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D52C2A56-7C6D-431B-8CC5-C0346323C1C6}">
+  <dimension ref="A1:B97"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1">
+        <v>131025</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1">
+        <v>118649</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="1">
+        <v>110029</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>329</v>
+      </c>
+      <c r="B5" s="1">
+        <v>103477</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" s="1">
+        <v>103167</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>414</v>
+      </c>
+      <c r="B7" s="1">
+        <v>99842</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>481</v>
+      </c>
+      <c r="B8" s="1">
+        <v>99165</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>482</v>
+      </c>
+      <c r="B9" s="1">
+        <v>99009</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="1">
+        <v>96805</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" s="1">
+        <v>96215</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>73</v>
+      </c>
+      <c r="B12" s="1">
+        <v>96138</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B13" s="1">
+        <v>96043</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1">
+        <v>95018</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>113</v>
+      </c>
+      <c r="B15" s="1">
+        <v>94543</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>181</v>
+      </c>
+      <c r="B16" s="1">
+        <v>93461</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>69</v>
+      </c>
+      <c r="B17" s="1">
+        <v>92826</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>60</v>
+      </c>
+      <c r="B18" s="1">
+        <v>92746</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="1">
+        <v>92293</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>483</v>
+      </c>
+      <c r="B20" s="1">
+        <v>91610</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" s="1">
+        <v>91438</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="1">
+        <v>90900</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>361</v>
+      </c>
+      <c r="B23" s="1">
+        <v>90457</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>190</v>
+      </c>
+      <c r="B24" s="1">
+        <v>89944</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>484</v>
+      </c>
+      <c r="B25" s="1">
+        <v>89685</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>371</v>
+      </c>
+      <c r="B26" s="1">
+        <v>89506</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>485</v>
+      </c>
+      <c r="B27" s="1">
+        <v>89430</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>53</v>
+      </c>
+      <c r="B28" s="1">
+        <v>88207</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>68</v>
+      </c>
+      <c r="B29" s="1">
+        <v>87856</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>81</v>
+      </c>
+      <c r="B30" s="1">
+        <v>87488</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>486</v>
+      </c>
+      <c r="B31" s="1">
+        <v>87033</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>487</v>
+      </c>
+      <c r="B32" s="1">
+        <v>86849</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>198</v>
+      </c>
+      <c r="B33" s="1">
+        <v>86504</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>40</v>
+      </c>
+      <c r="B34" s="1">
+        <v>86078</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>10</v>
+      </c>
+      <c r="B35" s="1">
+        <v>85708</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>488</v>
+      </c>
+      <c r="B36" s="1">
+        <v>85657</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>489</v>
+      </c>
+      <c r="B37" s="1">
+        <v>85638</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>18</v>
+      </c>
+      <c r="B38" s="1">
+        <v>85219</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>385</v>
+      </c>
+      <c r="B39" s="1">
+        <v>85089</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>27</v>
+      </c>
+      <c r="B40" s="1">
+        <v>82431</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>381</v>
+      </c>
+      <c r="B41" s="1">
+        <v>82399</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>354</v>
+      </c>
+      <c r="B42" s="1">
+        <v>81949</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>62</v>
+      </c>
+      <c r="B43" s="1">
+        <v>81840</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>195</v>
+      </c>
+      <c r="B44" s="1">
+        <v>81763</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>61</v>
+      </c>
+      <c r="B45" s="1">
+        <v>81696</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>26</v>
+      </c>
+      <c r="B46" s="1">
+        <v>81077</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>490</v>
+      </c>
+      <c r="B47" s="1">
+        <v>80594</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>491</v>
+      </c>
+      <c r="B48" s="1">
+        <v>80041</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>140</v>
+      </c>
+      <c r="B49" s="1">
+        <v>80025</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>492</v>
+      </c>
+      <c r="B50" s="1">
+        <v>79158</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>250</v>
+      </c>
+      <c r="B51" s="1">
+        <v>78569</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>332</v>
+      </c>
+      <c r="B52" s="1">
+        <v>77863</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>493</v>
+      </c>
+      <c r="B53" s="1">
+        <v>77851</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>39</v>
+      </c>
+      <c r="B54" s="1">
+        <v>77737</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>494</v>
+      </c>
+      <c r="B55" s="1">
+        <v>77575</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>173</v>
+      </c>
+      <c r="B56" s="1">
+        <v>77380</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>207</v>
+      </c>
+      <c r="B57" s="1">
+        <v>77158</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>435</v>
+      </c>
+      <c r="B58" s="1">
+        <v>76122</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
+        <v>19</v>
+      </c>
+      <c r="B59" s="1">
+        <v>75867</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
+        <v>92</v>
+      </c>
+      <c r="B60" s="1">
+        <v>75764</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>58</v>
+      </c>
+      <c r="B61" s="1">
+        <v>75281</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>495</v>
+      </c>
+      <c r="B62" s="1">
+        <v>75160</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>496</v>
+      </c>
+      <c r="B63" s="1">
+        <v>74813</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>5</v>
+      </c>
+      <c r="B64" s="1">
+        <v>74738</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
+        <v>141</v>
+      </c>
+      <c r="B65" s="1">
+        <v>74475</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
+        <v>77</v>
+      </c>
+      <c r="B66" s="1">
+        <v>74410</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
+        <v>178</v>
+      </c>
+      <c r="B67" s="1">
+        <v>73879</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>104</v>
+      </c>
+      <c r="B68" s="1">
+        <v>73747</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>424</v>
+      </c>
+      <c r="B69" s="1">
+        <v>73703</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>497</v>
+      </c>
+      <c r="B70" s="1">
+        <v>73540</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>498</v>
+      </c>
+      <c r="B71" s="1">
+        <v>73186</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
+        <v>65</v>
+      </c>
+      <c r="B72" s="1">
+        <v>72734</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>83</v>
+      </c>
+      <c r="B73" s="1">
+        <v>72596</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>100</v>
+      </c>
+      <c r="B74" s="1">
+        <v>71830</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>85</v>
+      </c>
+      <c r="B75" s="1">
+        <v>71752</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
+        <v>72</v>
+      </c>
+      <c r="B76" s="1">
+        <v>70462</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>41</v>
+      </c>
+      <c r="B77" s="1">
+        <v>69334</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>384</v>
+      </c>
+      <c r="B78" s="1">
+        <v>69192</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>79</v>
+      </c>
+      <c r="B79" s="1">
+        <v>68967</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>38</v>
+      </c>
+      <c r="B80" s="1">
+        <v>68682</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
+        <v>34</v>
+      </c>
+      <c r="B81" s="1">
+        <v>67544</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
+        <v>499</v>
+      </c>
+      <c r="B82" s="1">
+        <v>67536</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>55</v>
+      </c>
+      <c r="B83" s="1">
+        <v>67505</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
+        <v>500</v>
+      </c>
+      <c r="B84" s="1">
+        <v>66865</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>176</v>
+      </c>
+      <c r="B85" s="1">
+        <v>65217</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
+        <v>124</v>
+      </c>
+      <c r="B86" s="1">
+        <v>65013</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
+        <v>501</v>
+      </c>
+      <c r="B87" s="1">
+        <v>64837</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
+        <v>91</v>
+      </c>
+      <c r="B88" s="1">
+        <v>64459</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
+        <v>209</v>
+      </c>
+      <c r="B89" s="1">
+        <v>64413</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
+        <v>70</v>
+      </c>
+      <c r="B90" s="1">
+        <v>64133</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
+        <v>42</v>
+      </c>
+      <c r="B91" s="1">
+        <v>63833</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
+        <v>502</v>
+      </c>
+      <c r="B92" s="1">
+        <v>62865</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
+        <v>458</v>
+      </c>
+      <c r="B93" s="1">
+        <v>62004</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
+        <v>503</v>
+      </c>
+      <c r="B94" s="1">
+        <v>61162</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
+        <v>372</v>
+      </c>
+      <c r="B95" s="1">
+        <v>60393</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
+        <v>80</v>
+      </c>
+      <c r="B96" s="1">
+        <v>51590</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
+        <v>210</v>
+      </c>
+      <c r="B97" s="1">
+        <v>42790</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>